<commit_message>
fix(phase11): harden v1 corpus truth and integrity
</commit_message>
<xml_diff>
--- a/evals/corpus/v1/documents/duplicate-xlsx-002.xlsx
+++ b/evals/corpus/v1/documents/duplicate-xlsx-002.xlsx
@@ -415,6 +415,12 @@
   </sheetPr>
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -431,7 +437,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Brightline Retail</t>
+          <t>Harbor Hospitality</t>
         </is>
       </c>
     </row>
@@ -443,7 +449,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CUST-002</t>
+          <t>CUST-008</t>
         </is>
       </c>
     </row>
@@ -455,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PO-X-008</t>
+          <t>PO-X-010</t>
         </is>
       </c>
     </row>
@@ -467,7 +473,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -479,7 +485,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -503,10 +509,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Shared source bytes with the replay attempt.</t>
-        </is>
-      </c>
-    </row>
+          <t>Independent replay scenario with separate source identity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -532,20 +539,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SKU-029</t>
+          <t>SKU-021</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Visitor lanyard</t>
+          <t>Conference pad</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>14.00</t>
         </is>
       </c>
     </row>

</xml_diff>